<commit_message>
Correct 2T3X7 billet breakout
Co-authored-by: ScheelJW <ScheelJW@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/2T3_manning_detail.xlsx
+++ b/2T3_manning_detail.xlsx
@@ -16,628 +16,208 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>VM Response Totals (same basis as previous answer)</t>
+          <t>Email Table - 2T3X1 Mechanic / 2T3X7 Admin-Fleet Breakout</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>AFSC</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Skill Level</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Authorized</t>
-        </is>
-      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Current Assigned</t>
+          <t>Current Manning</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Current %</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Gains</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Losses</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
           <t>6 Months Out</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>6 Months %</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>2T3X1 - Mechanic</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>9-level</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1 authorized / 0 assigned - 0%</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>0%</t>
+          <t>1 authorized / 0 assigned - 0%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>2T3X1 - Mechanic</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>7-level</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6 authorized / 9 assigned - 150%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>150%</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>150%</t>
+          <t>6 authorized / 8 assigned - 133%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>2T3X1 - Mechanic</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>5-level</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>41</t>
-        </is>
-      </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>41 authorized / 19 assigned - 46%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>46%</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>34%</t>
+          <t>41 authorized / 15 assigned - 37%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>2T3X1 - Mechanic</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>3-level</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>13 authorized / 18 assigned - 138%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>138%</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>162%</t>
-        </is>
-      </c>
-    </row>
-    <row r="7"/>
+          <t>13 authorized / 21 assigned - 162%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2T3X7 - Admin/Fleet</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>7-level</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>3 authorized / 3 assigned - 100%</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>3 authorized / 4 assigned - 133%</t>
+        </is>
+      </c>
+    </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Breakout by AFSC Shred</t>
+          <t>2T3X7 - Admin/Fleet</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>5-level</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1 authorized / 1 assigned - 100%</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1 authorized / 0 assigned - 0%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>2T3X7 - Admin/Fleet</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Skill Level</t>
+          <t>3-level</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Authorized Billets</t>
+          <t>5 authorized / 7 assigned - 140%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Current Names</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Gains</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Losses</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>6 Months Out</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2T3X1 - Mechanic</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>9-level</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
+          <t>5 authorized / 7 assigned - 140%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2T3X1 - Mechanic</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>7-level</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t/>
+          <t>X1 authorized billets from AFMAA UMD Position. X7 authorized billets from visible X7 duty positions in AirmanGuardian because they were not represented as AD ENL X7 in the AFMAA position tab.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2T3X1 - Mechanic</t>
+          <t>Movement Window</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>5-level</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>41</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2T3X1 - Mechanic</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>3-level</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2T3X7 - Admin/Fleet</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>9-level</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>No AD ENL X7 billet found in UMD; current X7 names pulled from AirmanGuardian roster</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2T3X7 - Admin/Fleet</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>7-level</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>No AD ENL X7 billet found in UMD; current X7 names pulled from AirmanGuardian roster</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2T3X7 - Admin/Fleet</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>5-level</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>No AD ENL X7 billet found in UMD; current X7 names pulled from AirmanGuardian roster</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2T3X7 - Admin/Fleet</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>3-level</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>No AD ENL X7 billet found in UMD; current X7 names pulled from AirmanGuardian roster</t>
-        </is>
-      </c>
-    </row>
-    <row r="18"/>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Window</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Through 2026-11-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2T3X1 = mechanics; 2T3X7 = admin/fleet management.</t>
+          <t>Through 2026-11-30 from hail farewell.xlsx</t>
         </is>
       </c>
     </row>
@@ -753,7 +333,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -783,12 +363,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC; also listed as loss in hail/farewell</t>
+          <t>X1 billet/current count from UMD position sheet; also listed as loss</t>
         </is>
       </c>
     </row>
@@ -825,7 +405,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -855,12 +435,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -897,7 +477,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -927,12 +507,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -969,7 +549,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -999,12 +579,12 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -1041,7 +621,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1071,12 +651,12 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -1113,7 +693,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1143,12 +723,12 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -1185,7 +765,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1215,12 +795,12 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -1257,7 +837,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1287,12 +867,12 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -1329,7 +909,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1359,12 +939,12 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -1401,7 +981,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1431,12 +1011,12 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1053,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1503,12 +1083,12 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -1545,7 +1125,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1575,12 +1155,12 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -1617,7 +1197,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1647,12 +1227,12 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1269,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1719,12 +1299,12 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1341,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1791,12 +1371,12 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -1833,7 +1413,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1863,12 +1443,12 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -1905,7 +1485,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1935,12 +1515,12 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -1957,7 +1537,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2T331</t>
+          <t>2T351</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1977,7 +1557,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2007,12 +1587,12 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -2084,7 +1664,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Inbound by RNLTD within 6-month window</t>
+          <t>Inbound by RNLTD through 2026-11-30</t>
         </is>
       </c>
     </row>
@@ -2156,7 +1736,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Inbound by RNLTD within 6-month window</t>
+          <t>Inbound by RNLTD through 2026-11-30</t>
         </is>
       </c>
     </row>
@@ -2228,7 +1808,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Inbound by RNLTD within 6-month window</t>
+          <t>Inbound by RNLTD through 2026-11-30</t>
         </is>
       </c>
     </row>
@@ -2300,7 +1880,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Inbound by RNLTD within 6-month window</t>
+          <t>Inbound by RNLTD through 2026-11-30</t>
         </is>
       </c>
     </row>
@@ -2372,7 +1952,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Inbound by RNLTD within 6-month window</t>
+          <t>Inbound by RNLTD through 2026-11-30</t>
         </is>
       </c>
     </row>
@@ -2409,7 +1989,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2439,12 +2019,12 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC; also listed as loss in hail/farewell</t>
+          <t>X1 billet/current count from UMD position sheet; also listed as loss</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2061,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2511,12 +2091,12 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC; also listed as loss in hail/farewell</t>
+          <t>X1 billet/current count from UMD position sheet; also listed as loss</t>
         </is>
       </c>
     </row>
@@ -2553,7 +2133,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2583,12 +2163,12 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC; also listed as loss in hail/farewell</t>
+          <t>X1 billet/current count from UMD position sheet; also listed as loss</t>
         </is>
       </c>
     </row>
@@ -2625,7 +2205,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2655,12 +2235,12 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2277,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2727,12 +2307,12 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -2769,7 +2349,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2799,12 +2379,12 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2421,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2871,12 +2451,12 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -2913,7 +2493,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2943,12 +2523,12 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -2985,7 +2565,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3015,12 +2595,12 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -3057,7 +2637,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -3087,12 +2667,12 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -3129,7 +2709,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -3159,12 +2739,12 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -3201,7 +2781,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3231,12 +2811,12 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -3273,7 +2853,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3303,12 +2883,12 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -3345,7 +2925,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3375,12 +2955,12 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -3417,7 +2997,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3447,12 +3027,12 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3069,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3519,12 +3099,12 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3141,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3591,12 +3171,12 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -3633,7 +3213,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -3663,12 +3243,12 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -3705,7 +3285,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -3735,12 +3315,12 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -3812,7 +3392,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Inbound by RNLTD within 6-month window</t>
+          <t>Inbound by RNLTD through 2026-11-30</t>
         </is>
       </c>
     </row>
@@ -3849,7 +3429,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Not in detail current list</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -3884,7 +3464,7 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>Retirement/separation; listed here for visibility</t>
+          <t>Retirement/separation</t>
         </is>
       </c>
     </row>
@@ -3921,7 +3501,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Not in detail current list</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3956,7 +3536,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>PCS out; listed here for visibility</t>
+          <t>PCS out</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3573,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Not in detail current list</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -4028,7 +3608,7 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>Retirement/separation; listed here for visibility</t>
+          <t>Retirement/separation</t>
         </is>
       </c>
     </row>
@@ -4065,7 +3645,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -4095,12 +3675,12 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC; also listed as loss in hail/farewell</t>
+          <t>X1 billet/current count from UMD position sheet; also listed as loss</t>
         </is>
       </c>
     </row>
@@ -4137,7 +3717,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -4167,12 +3747,12 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -4209,7 +3789,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -4239,12 +3819,12 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -4281,7 +3861,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -4311,12 +3891,12 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -4353,7 +3933,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -4383,12 +3963,12 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -4425,7 +4005,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -4455,12 +4035,12 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -4497,7 +4077,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -4527,12 +4107,12 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -4569,7 +4149,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -4599,12 +4179,12 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -4641,7 +4221,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -4671,12 +4251,12 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -4708,12 +4288,12 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -4743,12 +4323,12 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -4780,12 +4360,12 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -4815,12 +4395,12 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -4852,12 +4432,12 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -4887,12 +4467,12 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -4924,12 +4504,12 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -4959,12 +4539,12 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -4996,12 +4576,12 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -5031,12 +4611,12 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -5068,12 +4648,12 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -5103,12 +4683,12 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -5140,12 +4720,12 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -5175,12 +4755,12 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -5217,7 +4797,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -5247,12 +4827,12 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet; also listed as loss in hail/farewell</t>
+          <t>X7 billet/current count from duty position roster; also listed as loss</t>
         </is>
       </c>
     </row>
@@ -5284,12 +4864,12 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -5319,12 +4899,12 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -5356,12 +4936,12 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -5391,12 +4971,12 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -5428,12 +5008,12 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -5463,12 +5043,12 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -5540,7 +5120,7 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>Inbound by RNLTD within 6-month window</t>
+          <t>Inbound by RNLTD through 2026-11-30</t>
         </is>
       </c>
     </row>
@@ -5656,7 +5236,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -5686,12 +5266,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC; also listed as loss in hail/farewell</t>
+          <t>X1 billet/current count from UMD position sheet; also listed as loss</t>
         </is>
       </c>
     </row>
@@ -5728,7 +5308,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -5758,12 +5338,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -5800,7 +5380,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -5830,12 +5410,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -5872,7 +5452,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -5902,12 +5482,12 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -5944,7 +5524,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -5974,12 +5554,12 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -6016,7 +5596,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -6046,12 +5626,12 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -6088,7 +5668,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -6118,12 +5698,12 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -6160,7 +5740,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -6190,12 +5770,12 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -6232,7 +5812,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -6262,12 +5842,12 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -6304,7 +5884,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -6334,12 +5914,12 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -6376,7 +5956,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -6406,12 +5986,12 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -6448,7 +6028,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -6478,12 +6058,12 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -6520,7 +6100,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -6550,12 +6130,12 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -6592,7 +6172,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -6622,12 +6202,12 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -6664,7 +6244,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -6694,12 +6274,12 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -6736,7 +6316,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -6766,12 +6346,12 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -6808,7 +6388,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -6838,12 +6418,12 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -6860,7 +6440,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2T331</t>
+          <t>2T351</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -6880,7 +6460,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -6910,12 +6490,12 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -6987,7 +6567,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Inbound by RNLTD within 6-month window</t>
+          <t>Inbound by RNLTD through 2026-11-30</t>
         </is>
       </c>
     </row>
@@ -7059,7 +6639,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Inbound by RNLTD within 6-month window</t>
+          <t>Inbound by RNLTD through 2026-11-30</t>
         </is>
       </c>
     </row>
@@ -7131,7 +6711,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Inbound by RNLTD within 6-month window</t>
+          <t>Inbound by RNLTD through 2026-11-30</t>
         </is>
       </c>
     </row>
@@ -7203,7 +6783,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Inbound by RNLTD within 6-month window</t>
+          <t>Inbound by RNLTD through 2026-11-30</t>
         </is>
       </c>
     </row>
@@ -7275,7 +6855,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Inbound by RNLTD within 6-month window</t>
+          <t>Inbound by RNLTD through 2026-11-30</t>
         </is>
       </c>
     </row>
@@ -7312,7 +6892,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -7342,12 +6922,12 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC; also listed as loss in hail/farewell</t>
+          <t>X1 billet/current count from UMD position sheet; also listed as loss</t>
         </is>
       </c>
     </row>
@@ -7384,7 +6964,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -7414,12 +6994,12 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC; also listed as loss in hail/farewell</t>
+          <t>X1 billet/current count from UMD position sheet; also listed as loss</t>
         </is>
       </c>
     </row>
@@ -7456,7 +7036,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -7486,12 +7066,12 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC; also listed as loss in hail/farewell</t>
+          <t>X1 billet/current count from UMD position sheet; also listed as loss</t>
         </is>
       </c>
     </row>
@@ -7528,7 +7108,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -7558,12 +7138,12 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -7600,7 +7180,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -7630,12 +7210,12 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -7672,7 +7252,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -7702,12 +7282,12 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -7744,7 +7324,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -7774,12 +7354,12 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7396,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -7846,12 +7426,12 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -7888,7 +7468,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -7918,12 +7498,12 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -7960,7 +7540,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -7990,12 +7570,12 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -8032,7 +7612,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -8062,12 +7642,12 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -8104,7 +7684,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -8134,12 +7714,12 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -8176,7 +7756,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -8206,12 +7786,12 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -8248,7 +7828,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -8278,12 +7858,12 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -8320,7 +7900,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -8350,12 +7930,12 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -8392,7 +7972,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -8422,12 +8002,12 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -8464,7 +8044,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -8494,12 +8074,12 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -8536,7 +8116,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -8566,12 +8146,12 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -8608,7 +8188,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -8638,12 +8218,12 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -8715,7 +8295,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Inbound by RNLTD within 6-month window</t>
+          <t>Inbound by RNLTD through 2026-11-30</t>
         </is>
       </c>
     </row>
@@ -8752,7 +8332,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Not in detail current list</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -8787,7 +8367,7 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>Retirement/separation; listed here for visibility</t>
+          <t>Retirement/separation</t>
         </is>
       </c>
     </row>
@@ -8824,7 +8404,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Not in detail current list</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -8859,7 +8439,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>PCS out; listed here for visibility</t>
+          <t>PCS out</t>
         </is>
       </c>
     </row>
@@ -8896,7 +8476,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Not in detail current list</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -8931,7 +8511,7 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>Retirement/separation; listed here for visibility</t>
+          <t>Retirement/separation</t>
         </is>
       </c>
     </row>
@@ -8968,7 +8548,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -8998,12 +8578,12 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC; also listed as loss in hail/farewell</t>
+          <t>X1 billet/current count from UMD position sheet; also listed as loss</t>
         </is>
       </c>
     </row>
@@ -9040,7 +8620,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -9070,12 +8650,12 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -9112,7 +8692,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -9142,12 +8722,12 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -9184,7 +8764,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -9214,12 +8794,12 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -9256,7 +8836,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -9286,12 +8866,12 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -9328,7 +8908,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -9358,12 +8938,12 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -9400,7 +8980,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -9430,12 +9010,12 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -9472,7 +9052,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -9502,12 +9082,12 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -9544,7 +9124,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Yes - UMD</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -9574,12 +9154,12 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AFMAA UMD Position</t>
+          <t>AFMAA UMD Position</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>Counted from UMD Control Skill Level 2 (Array); type from billet AFSC</t>
+          <t>X1 billet/current count from UMD position sheet</t>
         </is>
       </c>
     </row>
@@ -9690,12 +9270,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -9725,12 +9305,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -9762,12 +9342,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -9797,12 +9377,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -9834,12 +9414,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -9869,12 +9449,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -9906,12 +9486,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -9941,12 +9521,12 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -9978,12 +9558,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -10013,12 +9593,12 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -10050,12 +9630,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -10085,12 +9665,12 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -10122,12 +9702,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -10157,12 +9737,12 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -10199,7 +9779,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -10229,12 +9809,12 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet; also listed as loss in hail/farewell</t>
+          <t>X7 billet/current count from duty position roster; also listed as loss</t>
         </is>
       </c>
     </row>
@@ -10266,12 +9846,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -10301,12 +9881,12 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -10338,12 +9918,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -10373,12 +9953,12 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -10410,12 +9990,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Current roster</t>
+          <t>Current assigned</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Yes - roster</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -10445,12 +10025,12 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Export (15).xlsx / AirmanGuardian</t>
+          <t>AirmanGuardian</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>X7/admin current roster name; no AD ENL X7 billet found in UMD position sheet</t>
+          <t>X7 billet/current count from duty position roster</t>
         </is>
       </c>
     </row>
@@ -10522,7 +10102,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Inbound by RNLTD within 6-month window</t>
+          <t>Inbound by RNLTD through 2026-11-30</t>
         </is>
       </c>
     </row>

</xml_diff>